<commit_message>
Document 8473 30 80 vs 8414 59 conflict raised by MW freight agent
The forwarder's e-mail (ref 585427 / CZ26013469) describes the goods as
BRUSHLESS DC FAN under 8414599050. That does not match invoice
ISZ2680656:

- No occurrence of fan / 風扇 / ventilator / blower / motor anywhere in
  the invoice, packing list, marks, B/L or HBL.
- Per-piece net weights 0.415-0.614 kg are far above a server DC fan
  (0.05-0.20 kg) and consistent with metal heatsinks.
- 8414 59 90 has been invalid since 2006 (merged into 8414 59 80, later
  split into 8414 59 15/25/35/95).
- Had the goods been server fans, the correct code would be
  8414 59 15 00 at 0%, not 8414 59 95 at 2.3%.

Keeps 8473 30 80 00 and adds a sheet with the reasoning, plus two open
items: the truncated P70603-001 description and whether the e-mail
concerns a different consignment.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FzS4R76iGgmvV2mo8cyDu1
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Foxconn_CZ_ISZ2680656.xlsx
+++ b/output/HS_Code_Summary_Foxconn_CZ_ISZ2680656.xlsx
@@ -10,6 +10,7 @@
     <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Položky faktury" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Poznámky a kontroly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rozpor 8473 vs 8414" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -92,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -129,12 +130,9 @@
     <xf numFmtId="164" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -503,22 +501,22 @@
   <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" style="19" min="1" max="1"/>
+    <col width="18" customWidth="1" style="19" min="2" max="2"/>
+    <col width="44" customWidth="1" style="19" min="3" max="3"/>
+    <col width="44" customWidth="1" style="19" min="4" max="4"/>
+    <col width="10" customWidth="1" style="19" min="5" max="5"/>
+    <col width="18" customWidth="1" style="19" min="6" max="6"/>
+    <col width="12" customWidth="1" style="19" min="7" max="7"/>
+    <col width="16" customWidth="1" style="19" min="8" max="8"/>
+    <col width="16" customWidth="1" style="19" min="9" max="9"/>
+    <col width="15" customWidth="1" style="19" min="10" max="10"/>
+    <col width="8" customWidth="1" style="19" min="11" max="11"/>
+    <col width="14" customWidth="1" style="19" min="12" max="12"/>
+    <col width="60" customWidth="1" style="19" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46" customHeight="1">
+    <row r="1" ht="46" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Odesílatel (sender)</t>
@@ -640,7 +638,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>HS kód nebyl uveden na faktuře – odvozeno dle CCT/VPV KN (potvrzeno deklarací odesílatele 847330 na B/L). Clo 0 %. GW bez palet; +115,00 kg palety = 1 520,44 kg dle B/L.</t>
+          <t>HS kód nebyl uveden na faktuře – odvozeno dle CCT/VPV KN (potvrzeno deklarací odesílatele 847330 na B/L). Clo 0 %. GW bez palet; +115,00 kg palety = 1 520,44 kg dle B/L. ⚠️ E-mail MW uvádí 8414599050 / BRUSHLESS DC FAN – na toto zboží se nevztahuje (a kód je neplatný od 2006); viz list 'Rozpor 8473 vs 8414'.</t>
         </is>
       </c>
     </row>
@@ -748,20 +746,20 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="2"/>
+    <col width="40" customWidth="1" style="19" min="3" max="3"/>
+    <col width="16" customWidth="1" style="19" min="4" max="4"/>
+    <col width="13" customWidth="1" style="19" min="5" max="5"/>
+    <col width="14" customWidth="1" style="19" min="6" max="6"/>
+    <col width="14" customWidth="1" style="19" min="7" max="7"/>
+    <col width="13" customWidth="1" style="19" min="8" max="8"/>
+    <col width="17" customWidth="1" style="19" min="9" max="9"/>
+    <col width="30" customWidth="1" style="19" min="10" max="10"/>
+    <col width="14" customWidth="1" style="19" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="34" customHeight="1" s="19">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Customer P/N</t>
@@ -999,23 +997,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Hmotnost palet (pouze palety)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" s="11" t="inlineStr"/>
       <c r="G7" s="11" t="inlineStr"/>
       <c r="H7" s="12" t="inlineStr"/>
       <c r="I7" s="12" t="n">
         <v>115</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr"/>
@@ -1050,7 +1042,7 @@
   <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="170" customWidth="1" min="1" max="1"/>
+    <col width="170" customWidth="1" style="19" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1060,57 +1052,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Faktura č. ISZ2680656, datum odeslání 13-Aug-2026. AVC výdejka ILT2680069. P/O 4619002452.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Odesílatel (sender): ASIA VITAL COMPONENTS CO., LTD., West Industrial Park, Xinyang Community, Shajing Branch, Baoan District, Shenzhen 518104, CHINA.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Příjemce v ČR (consignee): FOXCONN CZ s.r.o. c/o JUSDA EUROPE, s.r.o. (HPE B/S for Foxconn), Ramps 100-121 GLS 100-121, Karlov 245, Kutná Hora 28401. EORI: CZ25938002. VAT (z faktury): CZ682138185.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Notify: Asia Vital Component Co., Ltd., New Taipei City, Taiwan.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Doprava: FANG ZHOU 27 / 260827N, Hong Kong → Hamburk (DE) → Kutná Hora. On board 29-Aug-2026. Kontejner OOLU9629630 / 40'HQ / plomba 30933593. CFS/CFS, telex release.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>B/L: HKGPRG2609004 (ref. ITMTPESE2609004), HBL Intermax 326081010. Doručení: Maurice Ward &amp; Co. s.r.o.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Balení: 7 palet / 134 kartonů, 7,670 CBM. Palety: c-煙燻棧板 = tepelně ošetřené (fumigované) palety s IPPC značením – doloženo na B/L ('SOLID WOOD MATERIAL WITH IPPC SEAL').</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="18">
         <f>== ⚠️ HS KÓD ODVOZEN – CCT/VPV KN tariff rule ===</f>
@@ -1118,85 +1108,83 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Faktura ani packing list NEOBSAHUJÍ HS kód u položek. HS kód byl odvozen metodou Společného celního sazebníku EU pro všechny 3 položky:</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t xml:space="preserve">  P70603-001 HF-Heatsink-DL360Perf Gen12 w → 8473 30 80 00</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t xml:space="preserve">  P70874-001 HF-HEATSINK-TOWER_4U_G12_STD → 8473 30 80 00</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t xml:space="preserve">  P51839-001 HF-散熱片成品4200 Gen11 STD → 8473 30 80 00</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>CO TO JE? Pasivní chladič (heatsink, 散熱片) – žebrovaný chladicí blok pro serverové CPU (HPE ProLiant DL360 Gen12, Tower 4U Gen12, 4200 Gen11).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Z ČEHO TO JE? Kov (hliník / měď, příp. s heat-pipe). POZOR: přesný materiál není v podkladech uveden – viz otevřené otázky níže.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>K ČEMU SLOUŽÍ? Odvod tepla z procesoru serveru; nemá vlastní funkci, je použitelné výhradně/hlavně se stroji č. 8471.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Postup nomenklaturou: Třída XVI → kapitola 84. Pozn. 2 písm. b) ke třídě XVI: části a součásti vhodné výhradně/hlavně pro určitý stroj se zařazují k tomuto stroji.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Číslo 8473 = části a součásti strojů čísel 8470–8472 → položka 8473 30 (části ADP strojů č. 8471) → 8473 30 80 (jiné než elektronické sestavy, chladič není osazená deska) → KN/TARIC 8473 30 80 00. Aplikována VPV KN 1 a 6.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Kontrolní shoda: odesílatel na B/L i HBL deklaruje 'HS CODE: 847330' a faktura je nadepsána 'PARTS OF COMPUTER USED ONLY' – odvozené zařazení se shoduje.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Smluvní sazba cla erga omnes pro 8473 30 80: 0 %.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="19" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="18">
         <f>== ⚠️ POPIS ZBOŽÍ – ŽÁDNÝ ČESKÝ POPIS NEDODÁN ===</f>
@@ -1204,29 +1192,27 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Klient NEDODAL český popis zboží a v podkladech (faktura, packing list, B/L, HBL, marks) není ŽÁDNÝ český text.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Ve sloupci 'Popis zboží – dle klienta' je proto ponechán původní popis klienta VERBATIM (angličtina / čínština).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Český popis ve vedlejším sloupci doplnil Maurice Ward pro potřeby JSD – NENÍ to popis klienta. Doporučuji si ho nechat od klienta potvrdit.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="19" t="inlineStr"/>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="18">
         <f>== CBAM ===</f>
@@ -1234,29 +1220,27 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>CBAM SE NEAPLIKUJE. KN 8473 30 80 není uvedeno v příloze I nařízení (EU) 2023/956 – CBAM se týká železa a oceli, hliníku, cementu, hnojiv, elektřiny a vodíku, nikoli částí ADP strojů.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>⚠️ Příjemce FOXCONN CZ s.r.o. (EORI CZ25938002) NENÍ v registru reference/CBAM_receivers_CZ.xlsx (list List1, 100 záznamů) – ani podle názvu firmy, ani podle EORI. Nenašel jsem ani JUSDA EUROPE s.r.o.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Pro tuto zásilku to nevadí (zboží není CBAM), ale doporučuji firmu prověřit a doplnit do registru pro případné budoucí zásilky s CBAM zbožím.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr"/>
-    </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="18">
         <f>== ANTIDUMPING ===</f>
@@ -1264,22 +1248,20 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Při zařazení do 8473 30 80 se antidumpingové clo NEUPLATŇUJE.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>⚠️ RIZIKO: pokud by celní orgán chladiče přeřadil mezi výrobky z hliníku (7616 99), uplatnilo by se antidumpingové clo na hliníkové výlisky/profily z ČLR (prov. nař. (EU) 2021/546) a zboží by zároveň spadlo pod CBAM. Zařazení do 8473 30 80 je podloženo tím, že jde o části použitelné výhradně pro servery č. 8471 – doporučuji mít po ruce technickou specifikaci / prohlášení výrobce o použití.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="19" t="inlineStr"/>
-    </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="18">
         <f>== PREFERENČNÍ PŮVOD / COO – KONTROLA DOKLADŮ ===</f>
@@ -1287,36 +1269,34 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>⚠️ PREFERENČNÍ VĚTA: NENALEZENA. Prošel jsem fakturu ISZ2680656, packing list, marks, B/L HKGPRG2609004 i HBL 326081010 – žádné prohlášení o preferenčním původu.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>⚠️ REX ČÍSLO: NA FAKTUŘE NENÍ. Faktura neobsahuje žádné REX číslo ani číslo celního povolení vývozce.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Původ zboží: ČÍNA (deklarováno na faktuře 'COUNTRY OF ORIGIN: CHINA', na packing listu i na obalových značkách 'MADE IN CHINA').</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>EU nemá s ČLR preferenční dohodu, proto by preferenční věta ani REX stejně nepřinesly zvýhodnění. Uplatňuje se sazba erga omnes = 0 % pro 8473 30 80, takže absence preferenčního dokladu NEMÁ v této zásilce dopad na clo.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="19" t="inlineStr"/>
-    </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="18">
         <f>== INCOTERM ===</f>
@@ -1324,29 +1304,27 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Incoterm dle faktury: DDP Kutná Hora (faktura, pole 'SHIPPING TERM: DDP' + poznámka 'DDP Kutna Hora VAT# CZ682138185'). Město je uvedeno.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>⚠️ NESOULAD V DOKLADECH: HBL Intermax 326081010 uvádí u zboží 'FOB HONG KONG' a 'FREIGHT COLLECT', zatímco B/L HKGPRG2609004 uvádí 'FREIGHT PREPAID'. Jde o přepravní podmínky mezi odesílatelem a dopravcem, ne o obchodní dodací doložku – pro celní účely platí DDP Kutná Hora z faktury. Doporučuji nesoulad potvrdit s odesílatelem.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>⚠️ DOPAD DDP NA CELNÍ HODNOTU: fakturovaná částka 66 634,68 USD je cena DDP Kutná Hora, tj. zahrnuje dopravu až do Kutné Hory, clo i případné poplatky. Pro celní hodnotu je nutné ODEČÍST náklady vzniklé po vstupu do EU (přeprava Hamburk → Kutná Hora) a clo/daně. Potřebuji od vás/od dopravce rozpis přepravních nákladů, abych celní hodnotu upravil – bez rozpisu je v tabulce uvedena plná fakturovaná hodnota.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr"/>
-    </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="18">
         <f>== SLEVA ===</f>
@@ -1354,15 +1332,13 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="19" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Na faktuře NENÍ uvedena žádná obchodní sleva – proporcionální rozpuštění slevy se proto neaplikovalo. Jednotkové ceny × množství přesně odpovídají celkové částce 66 634,68 USD.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="19" t="inlineStr"/>
-    </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="18">
         <f>== HMOTNOSTI – OVĚŘENÍ ===</f>
@@ -1370,36 +1346,34 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Čistá hmotnost 1 139,196 kg = 269,28 + 309,456 + 403,38 + 157,08 – souhlasí se součtem v packing listu.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="19" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Hrubá hmotnost položek 1 405,44 kg = 309,60 + 406,56 + 508,68 + 180,60. Palety 115,00 kg. Celkem 1 520,44 kg – souhlasí s B/L i HBL.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="19" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Množství 2 236 ks (760 + 504 + 972) – souhlasí s fakturou i packing listem.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="19" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Protože celá zásilka spadá pod jeden HS kód a jednoho odesílatele, je v souhrnu jeden řádek. Rozpad na položky je na listu 'Položky faktury'.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="19" t="inlineStr"/>
-    </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="18">
         <f>== ⚠️ OTEVŘENÉ OTÁZKY PRO KLIENTA ===</f>
@@ -1407,37 +1381,319 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>1) Český popis zboží – klient žádný nedodal. Potvrdit navržený český popis, nebo dodat vlastní.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="19" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>2) DDP – rozpis přepravních nákladů po vstupu do EU (Hamburk → Kutná Hora) pro úpravu celní hodnoty.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="19" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>3) Materiál chladičů (hliník / měď / heat-pipe) – pro obhájení zařazení 8473 30 80 vs. 7616 99 (antidumping + CBAM).</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="19" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>4) Název klienta a číslo zásilky pro pojmenování souboru – použil jsem Foxconn_CZ / ISZ2680656 (č. faktury). Dejte vědět, pokud používáte jiné označení.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="19" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>5) Nesoulad DDP (faktura) × FOB Hong Kong / freight collect (HBL) – potvrdit s odesílatelem.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="175" customWidth="1" style="19" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18">
+        <f>== ROZPOR: e-mail MW (8414599050 / BRUSHLESS DC FAN) × doklady k faktuře ISZ2680656 (HEATSINK) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E-mail Moniky Karlíkové (MW, ref. OR/Import/CZ26013469 / 585427 / HKG2026/08/14/1) uvádí zboží 'BRUSHLESS DC FAN (DC VENTILÁTOR)' a kód 8414599050.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>ZÁVĚR: pro zboží na faktuře ISZ2680656 je správně 8473 30 80 00. Kód 8414 59 se na toto zboží nevztahuje. Navíc kód 8414 59 90 50 z e-mailu NEEXISTUJE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>--- 1) V dokladech není ANI JEDNA zmínka o ventilátoru ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Prohledal jsem fakturu, packing list, list marks, B/L HKGPRG2609004 i HBL 326081010 na výrazy fan / 風扇 / 风扇 / ventilátor / blower / motor: NULA výskytů.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Popisy položek: 'HF-Heatsink-DL360Perf Gen12 w', 'HF-HEATSINK-TOWER_4U_G12_STD', 'HF-散熱片成品4200 Gen11 STD'. 散熱片 = chladicí žebro / chladič (heatsink), nikoli 風扇 (ventilátor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Faktura je nadepsána 'PARTS OF COMPUTER USED ONLY'. Odesílatel na obou konosamentech deklaruje 'HEATSINK' a 'HS CODE: 847330'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>--- 2) Hmotnost na kus vylučuje ventilátor ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>P70603-001: 11,220 kg / 20 ks = 0,561 kg/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P70874-001: 7,368 kg / 12 ks = 0,614 kg/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P51839-001: 7,470 kg / 18 ks = 0,415 kg/ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Serverový brushless DC ventilátor (40–80 mm) váží cca 0,05–0,20 kg/ks. Hmotnosti 0,42–0,61 kg/ks odpovídají kovovému chladiči (hliník/měď, příp. s heat-pipe), ne ventilátoru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>--- 3) Proč by u SKUTEČNÝCH ventilátorů 8473 správně NEBYLO ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pozn. 2 písm. a) ke třídě XVI má přednost před pozn. 2 písm. b): části, které jsou samy zbožím uvedeným v některém čísle kap. 84/85, se zařazují do svého vlastního čísla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ventilátor s vlastním motorem je zbožím čísla 8414, proto by patřil do 8414 59 i při použití výhradně v serveru – do 8473 30 by NEŠEL. Rozlišení je tedy věcné, ne formální.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Pasivní chladič naproti tomu vlastní číslo nemá → pozn. 2 písm. b) → 8473 30 80 (jiné než elektronické sestavy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>--- 4) Kód 8414 59 90 50 z e-mailu je neplatný ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CN 8414 59 90 byl sloučen do 8414 59 80 už v roce 2006; 8414 59 80 bylo později rozděleno. Platná struktura 2026: 8414 59 15 / 25 / 35 / 95.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8414 59 15 00 – ventilátory používané výhradně nebo hlavně k chlazení mikroprocesorů, telekomunikačních zařízení nebo zařízení pro automatizované zpracování dat – clo 0 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>8414 59 25 axiální / 8414 59 35 radiální / 8414 59 95 ostatní – clo 2,3 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Kdyby tedy skutečně šlo o serverové DC ventilátory, správný kód je 8414 59 15 00 (0 %), NIKOLI 8414 59 90 50 ani 8414 59 95 (2,3 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>--- 5) Dopad na clo ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>8473 30 80 00 = 0 % i 8414 59 15 00 = 0 % → mezi těmito dvěma kódy není rozdíl ve vyměřeném clu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Pozor ale na 8414 59 95 (2,3 %): z hodnoty 66 634,68 USD by to bylo cca 1 533 USD cla navíc. Chybný kód z e-mailu proto neopisovat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>--- 6) ⚠️ JEDINÁ OTEVŘENÁ VĚC: useknutý popis u P70603-001 ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Popis 'HF-Heatsink-DL360Perf Gen12 w' je v systému odesílatele useknutý na 29 znaků a končí na 'w' – může jít o 'w/ fan' (chladič s ventilátorem) i o něco jiného.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Pokud by šlo o sestavu chladič + ventilátor, zařazení by se řešilo dle VPV 3 b) podle podstatného charakteru a mohlo by spadnout do 8414 59 15 00 (rovněž 0 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Hmotnost 0,561 kg/ks a označení 'Perf' nicméně odpovídají pasivnímu výkonnostnímu chladiči pro 1U server (ventilátory šasi DL360 se dodávají jako samostatné díly).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>→ Vyžádat od AVC plný nezkrácený popis P70603-001. Do té doby ponechávám 8473 30 80 00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>--- 7) ⚠️ Jde vůbec o tutéž zásilku? ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>E-mail neuvádí číslo faktury ani B/L, takže vazbu na ISZ2680656 nelze z něj ověřit. Shoduje se příjemce (JUSDA Europe, Kutná Hora), původ HKG a datum 2026/08/14 (faktura 13-Aug-26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Monika Karlíková je zároveň kontaktem MW uvedeným na HBL 326081010 – stejný agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>NESEDÍ ale termín: 'Přijede na A1 Uhříněves cca 17/06' – naše zboží bylo naloženo on board až 29-Aug-2026, takže 17/06 nemůže platit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Kontejner je CFS/CFS (LCL konsolidace) a AVC vyrábí chladiče i ventilátory – e-mail se tedy patrně týká JINÉ zásilky AVC pro stejného příjemce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>→ Vyžádat od Moniky K. potvrzení, k jaké faktuře se ref. 585427 / CZ26013469 váže.</t>
         </is>
       </c>
     </row>

</xml_diff>